<commit_message>
Add ML scripts + cleaned tables
</commit_message>
<xml_diff>
--- a/Water_2109.xlsx
+++ b/Water_2109.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lisa-marieweidl/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lisa-marieweidl/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305566DF-098D-4C40-82F6-9171B64B2C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34B535E-DB8A-024C-9A95-FEC71BEDC754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="8" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$C$1:$C$823</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="44">
   <si>
     <t>PG31000292</t>
   </si>
@@ -145,9 +148,6 @@
     <t>AOX µg/l</t>
   </si>
   <si>
-    <t>n.a.</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -161,8 +161,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -247,7 +248,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -267,12 +268,39 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -582,18 +610,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:BBS823"/>
+  <dimension ref="A1:AH823"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:34" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>10</v>
@@ -13522,9 +13550,7 @@
       <c r="B154" s="3">
         <v>42850</v>
       </c>
-      <c r="C154" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="C154" s="1"/>
       <c r="D154" s="2">
         <v>9.5</v>
       </c>
@@ -22305,7 +22331,7 @@
       <c r="N254" s="2">
         <v>0.15</v>
       </c>
-      <c r="O254" s="2">
+      <c r="O254" s="8">
         <v>0</v>
       </c>
       <c r="P254" s="2">
@@ -41691,9 +41717,7 @@
       <c r="B482" s="3">
         <v>42858</v>
       </c>
-      <c r="C482" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="C482" s="1"/>
       <c r="D482" s="2">
         <v>7.8</v>
       </c>
@@ -48897,9 +48921,7 @@
       <c r="B566" s="3">
         <v>42852</v>
       </c>
-      <c r="C566" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="C566" s="1"/>
       <c r="D566" s="2">
         <v>7.9</v>
       </c>
@@ -65360,8 +65382,8 @@
       <c r="B756" s="3">
         <v>35940</v>
       </c>
-      <c r="C756" s="2">
-        <v>1010</v>
+      <c r="C756" s="7">
+        <v>10.1</v>
       </c>
       <c r="D756" s="2">
         <v>10.5</v>
@@ -69997,9 +70019,7 @@
       <c r="B811" s="3">
         <v>42864</v>
       </c>
-      <c r="C811" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="C811" s="1"/>
       <c r="D811" s="2">
         <v>10.8</v>
       </c>

</xml_diff>